<commit_message>
Overhaul DDMR to 5 digital transformation dimensions + add Messer demo
- Replace old dimensions (SL/FIN/IC) with ST/OSC/SM/TA/SC scored from
  digital transformation public signals with maturity labels
  (Legacy/Siloed/Strategic/Future Ready)
- Janatics composite updated to 64/100 (Siloed); Messer at 72/100 (Strategic)
- Add Next Best Actions section to web report, Word doc, and PowerPoint deck
  with initiative, expected benefit, cost of inaction, and why-now per company
- Login page updated to show two live demo cards (Janatics + Messer)
- Report page routes demo= param to correct dataset
- Regenerate xlsx, docx, pptx output files with new dimensions

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/Janatics_DDMR_Scorecard.xlsx
+++ b/output/Janatics_DDMR_Scorecard.xlsx
@@ -8,11 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorecard Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SL Detail" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SM Detail" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OSC Detail" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIN Detail" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC Detail" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ST Detail" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OSC Detail" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SM Detail" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA Detail" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SC Detail" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Index" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -101,19 +101,13 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="0000B050"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00FFC000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FF0000"/>
+      <color rgb="0000B050"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -141,7 +135,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000B050"/>
+        <fgColor rgb="00FFC000"/>
       </patternFill>
     </fill>
     <fill>
@@ -181,7 +175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -234,17 +228,14 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -338,7 +329,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>DDMR Dimension Scores</a:t>
+              <a:t>DDMR Digital Maturity — Dimension Scores</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -427,7 +418,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>SL Sub-Metric Scores</a:t>
+              <a:t>ST: Strategy — Sub-Metric Scores</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -442,7 +433,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'SL Detail'!D4</f>
+              <f>'ST Detail'!D4</f>
             </strRef>
           </tx>
           <spPr>
@@ -452,12 +443,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'SL Detail'!$B$5:$B$10</f>
+              <f>'ST Detail'!$B$5:$B$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'SL Detail'!$D$5:$D$10</f>
+              <f>'ST Detail'!$D$5:$D$9</f>
             </numRef>
           </val>
         </ser>
@@ -510,7 +501,90 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>SM Sub-Metric Scores</a:t>
+              <a:t>OSC: Operations &amp; Supply Chain — Sub-Metric Scores</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'OSC Detail'!D4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'OSC Detail'!$B$5:$B$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'OSC Detail'!$D$5:$D$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SM: Sales &amp; Marketing — Sub-Metric Scores</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -580,7 +654,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
@@ -593,7 +667,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>OSC Sub-Metric Scores</a:t>
+              <a:t>TA: Technology Adoption — Sub-Metric Scores</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -608,7 +682,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'OSC Detail'!D4</f>
+              <f>'TA Detail'!D4</f>
             </strRef>
           </tx>
           <spPr>
@@ -618,95 +692,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'OSC Detail'!$B$5:$B$9</f>
+              <f>'TA Detail'!$B$5:$B$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'OSC Detail'!$D$5:$D$9</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>FIN Sub-Metric Scores</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="bar"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'FIN Detail'!D4</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'FIN Detail'!$B$5:$B$10</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'FIN Detail'!$D$5:$D$10</f>
+              <f>'TA Detail'!$D$5:$D$9</f>
             </numRef>
           </val>
         </ser>
@@ -759,7 +750,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>IC Sub-Metric Scores</a:t>
+              <a:t>SC: Skills &amp; Capabilities — Sub-Metric Scores</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -774,7 +765,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'IC Detail'!D4</f>
+              <f>'SC Detail'!D4</f>
             </strRef>
           </tx>
           <spPr>
@@ -784,12 +775,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'IC Detail'!$B$5:$B$9</f>
+              <f>'SC Detail'!$B$5:$B$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'IC Detail'!$D$5:$D$9</f>
+              <f>'SC Detail'!$D$5:$D$9</f>
             </numRef>
           </val>
         </ser>
@@ -1284,11 +1275,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -1309,7 +1300,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>CIN: U31103TZ1991PTC003409   |   Report Date: 19 April 2026   |   Composite Score: 75.7/100</t>
+          <t>CIN: U31103TZ1991PTC003409   |   Report Date: 19 April 2026   |   Composite Score: 64/100   |   Maturity: Siloed</t>
         </is>
       </c>
     </row>
@@ -1317,13 +1308,13 @@
     <row r="6" ht="60" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>75.7</t>
+          <t>64</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>COMPOSITE DDMR SCORE
-(Weighted across 5 Dimensions)</t>
+          <t>COMPOSITE DDMR SCORE — Siloed
+(Weighted across 5 Digital Dimensions)</t>
         </is>
       </c>
     </row>
@@ -1350,122 +1341,122 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Rating</t>
+          <t>Maturity Level</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Strategy &amp; Leadership</t>
+          <t>Strategy</t>
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="E9" s="8" t="n">
-        <v>20.2</v>
+        <v>14</v>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Strategic</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Sales &amp; Marketing</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="n">
-        <v>78</v>
+          <t>Operations &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>65</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="E10" s="8" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="F10" s="10" t="inlineStr">
-        <is>
-          <t>Strong</t>
+      <c r="E10" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Siloed</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Operations &amp; Supply Chain</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="n">
-        <v>78</v>
+          <t>Sales &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>55</v>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="E11" s="8" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Strong</t>
+      <c r="E11" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Siloed</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="n">
-        <v>67</v>
+          <t>Technology Adoption</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>70</v>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="F12" s="12" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Strategic</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Industry Context</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="n">
-        <v>75</v>
+          <t>Skills &amp; Capabilities</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="n">
+        <v>60</v>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>Strong</t>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Siloed</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1467,7 @@
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>75.7</v>
+        <v>64</v>
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
@@ -1484,11 +1475,11 @@
         </is>
       </c>
       <c r="E14" s="14" t="n">
-        <v>75.7</v>
+        <v>64</v>
       </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Siloed</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E11"/>
+  <dimension ref="B2:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1536,7 +1527,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SL — Strategy &amp; Leadership   |   Score: 81/100   |   Weight: 25%</t>
+          <t>ST — Strategy   |   Score: 70/100   |   Weight: 20%   |   Strategic</t>
         </is>
       </c>
     </row>
@@ -1558,147 +1549,127 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Evidence / Rationale</t>
+          <t>Public Signal / Evidence</t>
         </is>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>SL01</t>
+          <t>ST01</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>Founder/Company Tenure (est. 1977, 49 yrs)</t>
+          <t>Digital Strategy Articulation</t>
         </is>
       </c>
       <c r="D5" s="17" t="n">
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>Founded 1977; incorporated 1991 — one of India's oldest domestic pneumatics brands</t>
+          <t>I4.0 and digital products mentioned but no formal DX roadmap publicly disclosed</t>
         </is>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>SL02</t>
+          <t>ST02</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>Director Profile &amp; DIN Compliance</t>
-        </is>
-      </c>
-      <c r="D6" s="17" t="n">
-        <v>75</v>
+          <t>Leadership Technology Vision</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="n">
+        <v>72</v>
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>3 active directors: G Jaganathan, GC Nageswaran, R Ramesh — all DINs active</t>
+          <t>Management pivoted to electric actuators, robotics, sensors — signals digital awareness</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>SL03</t>
+          <t>ST03</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Governance &amp; Filing Compliance</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="n">
-        <v>80</v>
+          <t>Digital Investment Signals</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>75</v>
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>AGM held Sept 30 2024; filings current with ROC Coimbatore</t>
+          <t>New IoT-enabled product lines indicate technology capex commitment</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>SL04</t>
+          <t>ST04</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>Debt &amp; Charge Structure</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="n">
-        <v>78</v>
+          <t>Technology Partnerships</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>68</v>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>ICRA-rated; stable outlook; healthy debt protection metrics per ICRA rationale</t>
+          <t>DSIR R&amp;D recognition confirmed; no public tech alliance or digital ecosystem partnerships</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>SL05</t>
+          <t>ST05</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>Strategic Direction &amp; Diversification</t>
-        </is>
-      </c>
-      <c r="D9" s="17" t="n">
-        <v>82</v>
+          <t>Innovation Pipeline</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="n">
+        <v>70</v>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>Expanded beyond pneumatics → electric actuators, robotics, Industry 4.0 alignment</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>SL06</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="inlineStr">
-        <is>
-          <t>Global Presence &amp; Export Strategy</t>
-        </is>
-      </c>
-      <c r="D10" s="17" t="n">
-        <v>88</v>
-      </c>
-      <c r="E10" s="16" t="inlineStr">
-        <is>
-          <t>Operations in 42+ countries; subsidiaries in USA and Germany; global distribution network</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="18" t="inlineStr">
+          <t>Incremental product digitization underway; no IP filing trail or open innovation signals</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>AVG</t>
         </is>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>Dimension Average Score</t>
         </is>
       </c>
-      <c r="D11" s="18" t="n">
-        <v>81</v>
-      </c>
-      <c r="E11" s="19" t="inlineStr">
-        <is>
-          <t>Weighted contribution to composite: 20.2 pts</t>
+      <c r="D10" s="19" t="n">
+        <v>70</v>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Maturity: Strategic  |  Weighted contribution: 14.0 pts</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1701,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SM — Sales &amp; Marketing   |   Score: 78/100   |   Weight: 20%</t>
+          <t>OSC — Operations &amp; Supply Chain   |   Score: 65/100   |   Weight: 20%   |   Siloed</t>
         </is>
       </c>
     </row>
@@ -1752,127 +1723,127 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Evidence / Rationale</t>
+          <t>Public Signal / Evidence</t>
         </is>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>SM01</t>
+          <t>OSC01</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>Revenue Growth vs Industry CAGR</t>
-        </is>
-      </c>
-      <c r="D5" s="20" t="n">
-        <v>55</v>
+          <t>Digital Manufacturing Readiness</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="n">
+        <v>60</v>
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>Revenue grew ~4-5% YoY (FY24→FY25) vs industry CAGR of 6.9% — slightly below market</t>
+          <t>70,000 sqm Coimbatore plant with CNC; no Industry 4.0 certification or smart factory disclosure</t>
         </is>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>SM02</t>
+          <t>OSC02</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>Revenue Scale</t>
+          <t>Supply Chain Visibility Tools</t>
         </is>
       </c>
       <c r="D6" s="17" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>FY2025 revenue: ₹531 Cr (~$63M USD) — significant scale for domestic manufacturer</t>
+          <t>No public disclosure of ERP, SCM platform, or supply chain digitization initiative</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>SM03</t>
+          <t>OSC03</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Customer Diversity</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="n">
-        <v>90</v>
+          <t>Process Automation Adoption</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>70</v>
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>17,000+ customers across pharma, auto, packaging, printing, food, medical, textile</t>
+          <t>CNC machining, casting automation, surface treatment lines — physical automation established</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>SM04</t>
+          <t>OSC04</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>Distribution Network</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="n">
-        <v>85</v>
+          <t>Quality Management (Digital)</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>72</v>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>200 distribution partners globally; 3 plants for regional coverage</t>
+          <t>ICRA notes consistent regulatory compliance; ISO quality system assumed but unconfirmed</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>SM05</t>
+          <t>OSC05</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>Brand Strength</t>
-        </is>
-      </c>
-      <c r="D9" s="17" t="n">
-        <v>80</v>
+          <t>Industry 4.0 Integration</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="n">
+        <v>73</v>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>49-year brand; own-label (Janatics); member of AIA India; DSIR-recognized R&amp;D</t>
+          <t>I4.0 product portfolio exists; internal I4.0 adoption for own manufacturing not disclosed</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>AVG</t>
         </is>
       </c>
-      <c r="C10" s="19" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>Dimension Average Score</t>
         </is>
       </c>
-      <c r="D10" s="18" t="n">
-        <v>78</v>
-      </c>
-      <c r="E10" s="19" t="inlineStr">
-        <is>
-          <t>Weighted contribution to composite: 15.6 pts</t>
+      <c r="D10" s="19" t="n">
+        <v>65</v>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Maturity: Siloed  |  Weighted contribution: 13.0 pts</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1875,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>OSC — Operations &amp; Supply Chain   |   Score: 78/100   |   Weight: 20%</t>
+          <t>SM — Sales &amp; Marketing   |   Score: 55/100   |   Weight: 20%   |   Siloed</t>
         </is>
       </c>
     </row>
@@ -1926,127 +1897,127 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Evidence / Rationale</t>
+          <t>Public Signal / Evidence</t>
         </is>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>OSC01</t>
+          <t>SM01</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>Manufacturing Scale &amp; Capacity</t>
+          <t>Digital Presence &amp; SEO</t>
         </is>
       </c>
       <c r="D5" s="17" t="n">
-        <v>85</v>
+        <v>60</v>
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>70,000 sqm facility in Coimbatore; additional plants in Ahmedabad and Noida</t>
+          <t>Two product websites (janatics.com, janaticspneumatics.com); SEO signals moderate</t>
         </is>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>OSC02</t>
+          <t>SM02</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>Product Portfolio Breadth</t>
+          <t>Social Media Engagement</t>
         </is>
       </c>
       <c r="D6" s="17" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>3,500+ distinct products across pneumatics, vacuum, hydraulics, didactics, robotics</t>
+          <t>Limited LinkedIn activity signal; no active social media marketing evidenced</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>OSC03</t>
+          <t>SM03</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>R&amp;D &amp; Technology Capability</t>
+          <t>E-commerce / Digital Ordering</t>
         </is>
       </c>
       <c r="D7" s="17" t="n">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>DSIR-recognized R&amp;D division; CNC machining; casting operations; expanding to robotics</t>
+          <t>No evidence of digital ordering portal, e-catalog with pricing, or B2B e-commerce</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>OSC04</t>
+          <t>SM04</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>GST &amp; Regulatory Compliance</t>
-        </is>
-      </c>
-      <c r="D8" s="20" t="n">
-        <v>72</v>
+          <t>Digital Marketing Activity</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>55</v>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>Active GST entity; ICRA notes consistent compliance; e-Invoice enablement assumed</t>
+          <t>Web presence established; no paid digital campaigns or content marketing evidenced</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>OSC05</t>
+          <t>SM05</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>Supply Chain Digitization</t>
-        </is>
-      </c>
-      <c r="D9" s="20" t="n">
-        <v>65</v>
+          <t>CRM &amp; Customer Data Utilization</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="n">
+        <v>75</v>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>Industry 4.0 product range signals awareness; internal digitization not publicly quantified</t>
+          <t>17,000+ customers across 7 industries — implies structured data; CRM platform undisclosed</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>AVG</t>
         </is>
       </c>
-      <c r="C10" s="19" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>Dimension Average Score</t>
         </is>
       </c>
-      <c r="D10" s="18" t="n">
-        <v>78</v>
-      </c>
-      <c r="E10" s="19" t="inlineStr">
-        <is>
-          <t>Weighted contribution to composite: 15.6 pts</t>
+      <c r="D10" s="19" t="n">
+        <v>55</v>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Maturity: Siloed  |  Weighted contribution: 11.0 pts</t>
         </is>
       </c>
     </row>
@@ -2065,7 +2036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E11"/>
+  <dimension ref="B2:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2078,7 +2049,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>FIN — Finance   |   Score: 67/100   |   Weight: 25%</t>
+          <t>TA — Technology Adoption   |   Score: 70/100   |   Weight: 20%   |   Strategic</t>
         </is>
       </c>
     </row>
@@ -2100,147 +2071,127 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Evidence / Rationale</t>
+          <t>Public Signal / Evidence</t>
         </is>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>FIN01</t>
+          <t>TA01</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>Revenue Scale (₹531 Cr FY25)</t>
+          <t>Website &amp; Digital Infrastructure</t>
         </is>
       </c>
       <c r="D5" s="17" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>₹531 Cr revenue — strong for unlisted domestic manufacturer in pneumatics segment</t>
+          <t>Functional product websites; no modern tech stack, API integrations, or customer portal evidence</t>
         </is>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>FIN02</t>
+          <t>TA02</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>Revenue Growth Rate (4% YoY)</t>
-        </is>
-      </c>
-      <c r="D6" s="20" t="n">
-        <v>55</v>
+          <t>IoT / Smart Product Portfolio</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="n">
+        <v>80</v>
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>FY24: ₹507.9 Cr → FY25: ₹527.8 Cr — 4% growth; steady but below industry pace</t>
+          <t>Electric actuators, smart sensors, robotics, I4.0 didactic equipment launched — strong product digitization</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>FIN03</t>
+          <t>TA03</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>EBITDA Trajectory</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="n">
-        <v>42</v>
+          <t>Cloud &amp; SaaS Adoption</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="n">
+        <v>60</v>
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>EBITDA CAGR -22% (1-yr) — margin compression flagged; needs monitoring</t>
+          <t>No public disclosures of cloud migration, SaaS tools, or digital collaboration platforms</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>FIN04</t>
+          <t>TA04</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>Credit Profile (ICRA Rated)</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="n">
-        <v>82</v>
+          <t>R&amp;D in Digital / Smart Tech</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>78</v>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>ICRA rated with stable outlook; multiple reaffirmations; healthy debt protection metrics</t>
+          <t>DSIR R&amp;D actively developing robotic systems, sensor products, and smart automation equipment</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>FIN05</t>
+          <t>TA05</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>Capital Structure</t>
-        </is>
-      </c>
-      <c r="D9" s="17" t="n">
-        <v>75</v>
+          <t>Cybersecurity &amp; Data Practices</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="n">
+        <v>67</v>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>Auth. capital ₹30 Cr; paid-up ₹26.5 Cr; nearly fully subscribed — conservative but sound</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>FIN06</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="inlineStr">
-        <is>
-          <t>Employee Productivity</t>
-        </is>
-      </c>
-      <c r="D10" s="20" t="n">
+          <t>ICRA-compliant practices; no public cybersecurity framework, ISO 27001, or data policy disclosed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>AVG</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>Dimension Average Score</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="n">
         <v>70</v>
       </c>
-      <c r="E10" s="16" t="inlineStr">
-        <is>
-          <t>₹531 Cr / 662 employees = ₹80L per employee — decent for manufacturing sector</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>AVG</t>
-        </is>
-      </c>
-      <c r="C11" s="19" t="inlineStr">
-        <is>
-          <t>Dimension Average Score</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="n">
-        <v>67</v>
-      </c>
-      <c r="E11" s="19" t="inlineStr">
-        <is>
-          <t>Weighted contribution to composite: 16.8 pts</t>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Maturity: Strategic  |  Weighted contribution: 14.0 pts</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2223,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>IC — Industry Context   |   Score: 75/100   |   Weight: 10%</t>
+          <t>SC — Skills &amp; Capabilities   |   Score: 60/100   |   Weight: 20%   |   Siloed</t>
         </is>
       </c>
     </row>
@@ -2294,127 +2245,127 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Evidence / Rationale</t>
+          <t>Public Signal / Evidence</t>
         </is>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>IC01</t>
+          <t>SC01</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>India Pneumatics Market Size</t>
-        </is>
-      </c>
-      <c r="D5" s="20" t="n">
-        <v>70</v>
+          <t>Digital Talent Hiring Signals</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="n">
+        <v>55</v>
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>India pneumatics market ~$1.06B (2024); growing to $1.94B by 2033 — mid-size TAM</t>
+          <t>662 employees primarily engineering/manufacturing; limited signals of software or data roles hired</t>
         </is>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>IC02</t>
+          <t>SC02</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>Industry Growth Rate (6.9% CAGR)</t>
-        </is>
-      </c>
-      <c r="D6" s="17" t="n">
-        <v>78</v>
+          <t>Technical Workforce Depth</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="n">
+        <v>72</v>
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>India pneumatic equipment CAGR 6.9% (2025–2033); aligned with industrial capex cycle</t>
+          <t>Strong mechanical and manufacturing engineering talent; DSIR R&amp;D team; CNC and automation specialists</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>IC03</t>
+          <t>SC03</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Competitive Position</t>
-        </is>
-      </c>
-      <c r="D7" s="20" t="n">
-        <v>70</v>
+          <t>Digital Training Programs</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="n">
+        <v>50</v>
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>Domestic brand competing with global leaders (SMC, Festo, Parker); strong in mid-market</t>
+          <t>No public evidence of L&amp;D investment, digital upskilling programs, or online learning adoption</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>IC04</t>
+          <t>SC04</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>Macro Tailwinds</t>
+          <t>Leadership Digital Literacy</t>
         </is>
       </c>
       <c r="D8" s="17" t="n">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>Make in India, PLI schemes, manufacturing automation, China+1 strategy all favourable</t>
+          <t>Management demonstrates I4.0 awareness via product decisions; no DX leadership hire signals</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>IC05</t>
+          <t>SC05</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>End-Market Diversification</t>
+          <t>Innovation Culture Signals</t>
         </is>
       </c>
       <c r="D9" s="17" t="n">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>6+ industries: pharma, auto, packaging, food, medical, textile — low single-sector risk</t>
+          <t>DSIR R&amp;D present; no public hackathon, innovation lab, or employee innovation program signals</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>AVG</t>
         </is>
       </c>
-      <c r="C10" s="19" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>Dimension Average Score</t>
         </is>
       </c>
-      <c r="D10" s="18" t="n">
-        <v>75</v>
-      </c>
-      <c r="E10" s="19" t="inlineStr">
-        <is>
-          <t>Weighted contribution to composite: 7.5 pts</t>
+      <c r="D10" s="19" t="n">
+        <v>60</v>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Maturity: Siloed  |  Weighted contribution: 12.0 pts</t>
         </is>
       </c>
     </row>
@@ -2433,7 +2384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E31"/>
+  <dimension ref="B2:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2444,43 +2395,43 @@
   </cols>
   <sheetData>
     <row r="2" ht="24" customHeight="1">
-      <c r="B2" s="22" t="inlineStr">
-        <is>
-          <t>Evidence Index — Janatics India Private Limited</t>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>Evidence Index — Janatics India Private Limited — Digital Diagnostic and Maturity Report</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>Sub-Metric</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
-        <is>
-          <t>Evidence</t>
+      <c r="E4" s="19" t="inlineStr">
+        <is>
+          <t>Public Signal / Evidence</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>SL01</t>
+          <t>ST01</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>Founder/Company Tenure</t>
+          <t>Digital Strategy Articulation</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">
@@ -2490,85 +2441,85 @@
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>Incorporated 1991; brand established 1977 — 49-year operating history</t>
+          <t>No formal DX roadmap in public disclosures; I4.0 product lines signal intent</t>
         </is>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>SL02</t>
+          <t>ST02</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>Director Profile</t>
+          <t>Leadership Technology Vision</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>MCA public records</t>
+          <t>Janatics website</t>
         </is>
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>3 active directors; AGM Sept 2024; ROC Coimbatore filings current</t>
+          <t>Management added electric actuators, robotics, smart sensors — visible strategic pivot</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>SL03</t>
+          <t>ST03</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Governance Compliance</t>
+          <t>Digital Investment Signals</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>MCA / Zaubacorp</t>
+          <t>Janatics website / ICRA</t>
         </is>
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>Annual filings current; AGM held within statutory deadline</t>
+          <t>New IoT-enabled product categories launched; DSIR R&amp;D investment ongoing</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>SL04</t>
+          <t>ST04</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>Debt Structure</t>
+          <t>Technology Partnerships</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>ICRA Rationale Report</t>
+          <t>MCA / Public records</t>
         </is>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>ICRA rated; stable outlook; healthy debt protection metrics; multiple reaffirmations</t>
+          <t>DSIR R&amp;D confirmed; no public digital alliance, co-development, or tech partner disclosures</t>
         </is>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>SL05</t>
+          <t>ST05</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>Strategic Direction</t>
+          <t>Innovation Pipeline</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
@@ -2578,19 +2529,19 @@
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>Expanded to electric actuators, sensors, motors, robotics — Industry 4.0 pivot</t>
+          <t>Incremental product digitization; no IP filing, open innovation, or startup engagement public</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>SL06</t>
+          <t>OSC01</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>Global Presence</t>
+          <t>Digital Manufacturing Readiness</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
@@ -2600,415 +2551,415 @@
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>42+ countries; subsidiaries USA and Germany; 200 global distribution partners</t>
+          <t>70,000 sqm Coimbatore plant; CNC machining; no I4.0 certification or smart factory claims</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>SM01</t>
+          <t>OSC02</t>
         </is>
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>Revenue Growth</t>
+          <t>Supply Chain Visibility Tools</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>ICRA / Tracxn</t>
+          <t>Public records</t>
         </is>
       </c>
       <c r="E11" s="16" t="inlineStr">
         <is>
-          <t>FY24: ₹507.9 Cr → FY25: ₹527.8 Cr; ~4% YoY vs 6.9% industry CAGR</t>
+          <t>No ERP, SCM platform, or supply chain digitization initiative disclosed publicly</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>SM02</t>
+          <t>OSC03</t>
         </is>
       </c>
       <c r="C12" s="16" t="inlineStr">
         <is>
-          <t>Revenue Scale</t>
+          <t>Process Automation Adoption</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>Tracxn / ICRA 2025</t>
+          <t>janaticspneumatics.com</t>
         </is>
       </c>
       <c r="E12" s="16" t="inlineStr">
         <is>
-          <t>₹531 Cr FY2025; consistent ₹500 Cr+ revenue for 2 consecutive years</t>
+          <t>CNC machining centers, casting, surface treatment — physical automation well established</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>SM03</t>
+          <t>OSC04</t>
         </is>
       </c>
       <c r="C13" s="16" t="inlineStr">
         <is>
-          <t>Customer Diversity</t>
+          <t>Quality Management (Digital)</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>Janatics website</t>
+          <t>ICRA Rationale</t>
         </is>
       </c>
       <c r="E13" s="16" t="inlineStr">
         <is>
-          <t>17,000+ customers; 6+ industries: pharma, auto, packaging, food, medical, textile</t>
+          <t>ICRA notes consistent compliance; ISO quality framework assumed but not confirmed publicly</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>SM04</t>
+          <t>OSC05</t>
         </is>
       </c>
       <c r="C14" s="16" t="inlineStr">
         <is>
-          <t>Distribution Network</t>
+          <t>Industry 4.0 Integration</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>janaticspneumatics.com</t>
+          <t>Janatics website</t>
         </is>
       </c>
       <c r="E14" s="16" t="inlineStr">
         <is>
-          <t>200 global distribution partners; 3 manufacturing plants for regional reach</t>
+          <t>I4.0 didactic product line exists; internal adoption for own operations undisclosed</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>SM05</t>
+          <t>SM01</t>
         </is>
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>Brand Strength</t>
+          <t>Digital Presence &amp; SEO</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>AIA India / DSIR</t>
+          <t>janatics.com / janaticspneumatics.com</t>
         </is>
       </c>
       <c r="E15" s="16" t="inlineStr">
         <is>
-          <t>Member of Automation Industry Association India; DSIR-recognized R&amp;D division</t>
+          <t>Two product websites with online catalog; SEO signals moderate; no chatbot or digital engagement tools</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>OSC01</t>
+          <t>SM02</t>
         </is>
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>Manufacturing Scale</t>
+          <t>Social Media Engagement</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>janaticspneumatics.com</t>
+          <t>LinkedIn / Public</t>
         </is>
       </c>
       <c r="E16" s="16" t="inlineStr">
         <is>
-          <t>70,000 sqm Coimbatore HQ; additional Ahmedabad and Noida plants</t>
+          <t>Limited LinkedIn activity signal; no active social media marketing strategy evidenced</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>OSC02</t>
+          <t>SM03</t>
         </is>
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>Product Portfolio</t>
+          <t>E-commerce / Digital Ordering</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>ICRA Rationale</t>
+          <t>Public research</t>
         </is>
       </c>
       <c r="E17" s="16" t="inlineStr">
         <is>
-          <t>3,500+ distinct products across pneumatics, vacuum, hydraulics, didactics, robotics</t>
+          <t>No B2B e-commerce, digital ordering portal, or online pricing catalog identified</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>OSC03</t>
+          <t>SM04</t>
         </is>
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>R&amp;D Capability</t>
+          <t>Digital Marketing Activity</t>
         </is>
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
-          <t>DSIR / Janatics website</t>
+          <t>Web / Public</t>
         </is>
       </c>
       <c r="E18" s="16" t="inlineStr">
         <is>
-          <t>DSIR-recognized R&amp;D; CNC and casting; expanding to robotic systems</t>
+          <t>Websites established; no evidence of paid search, content marketing, or digital ad activity</t>
         </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>OSC04</t>
+          <t>SM05</t>
         </is>
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>GST Compliance</t>
+          <t>CRM &amp; Customer Data</t>
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
-          <t>ICRA / public records</t>
+          <t>Janatics / ICRA</t>
         </is>
       </c>
       <c r="E19" s="16" t="inlineStr">
         <is>
-          <t>Active GST entity; ICRA notes consistent regulatory compliance</t>
+          <t>17,000+ customers across 7 industries implies structured data management; CRM tool undisclosed</t>
         </is>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>OSC05</t>
+          <t>TA01</t>
         </is>
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>Digitization</t>
+          <t>Website &amp; Digital Infrastructure</t>
         </is>
       </c>
       <c r="D20" s="16" t="inlineStr">
         <is>
-          <t>Janatics website</t>
+          <t>janatics.com</t>
         </is>
       </c>
       <c r="E20" s="16" t="inlineStr">
         <is>
-          <t>Industry 4.0 product line exists; internal ERP/digitization not publicly disclosed</t>
+          <t>Functional websites; no evidence of modern CMS, API layer, or customer self-service portal</t>
         </is>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>FIN01</t>
+          <t>TA02</t>
         </is>
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>Revenue FY2025</t>
+          <t>IoT / Smart Product Portfolio</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr">
         <is>
-          <t>ICRA Rationale 2025</t>
+          <t>Janatics website / ICRA</t>
         </is>
       </c>
       <c r="E21" s="16" t="inlineStr">
         <is>
-          <t>FY2025 revenue: ₹527.8 Cr (ICRA) / ₹531 Cr (Tracxn)</t>
+          <t>Electric actuators, smart sensors, robotic systems, I4.0 didactics — strong product-layer digitization</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>FIN02</t>
+          <t>TA03</t>
         </is>
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>Revenue Growth</t>
+          <t>Cloud &amp; SaaS Adoption</t>
         </is>
       </c>
       <c r="D22" s="16" t="inlineStr">
         <is>
-          <t>ICRA</t>
+          <t>Public records</t>
         </is>
       </c>
       <c r="E22" s="16" t="inlineStr">
         <is>
-          <t>4% YoY growth FY24→FY25; 3-yr CAGR not publicly available</t>
+          <t>No public cloud migration, SaaS adoption, or digital collaboration platform disclosures found</t>
         </is>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="B23" s="15" t="inlineStr">
         <is>
-          <t>FIN03</t>
+          <t>TA04</t>
         </is>
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>EBITDA Trajectory</t>
+          <t>R&amp;D in Digital / Smart Tech</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
         <is>
-          <t>Tracxn</t>
+          <t>DSIR / Janatics website</t>
         </is>
       </c>
       <c r="E23" s="16" t="inlineStr">
         <is>
-          <t>EBITDA CAGR -22% (1-year) — margin compression; specific % not disclosed</t>
+          <t>DSIR-recognized R&amp;D developing robotic systems, sensor products, and smart automation equipment</t>
         </is>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>FIN04</t>
+          <t>TA05</t>
         </is>
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>Credit Profile</t>
+          <t>Cybersecurity &amp; Data Practices</t>
         </is>
       </c>
       <c r="D24" s="16" t="inlineStr">
         <is>
-          <t>ICRA</t>
+          <t>ICRA / Public</t>
         </is>
       </c>
       <c r="E24" s="16" t="inlineStr">
         <is>
-          <t>Stable outlook; healthy credit; multiple reaffirmations over 3+ years</t>
+          <t>ICRA-compliant; no public cybersecurity framework, ISO 27001 certification, or data policy found</t>
         </is>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>FIN05</t>
+          <t>SC01</t>
         </is>
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>Capital Structure</t>
+          <t>Digital Talent Hiring Signals</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
-          <t>MCA / Zaubacorp</t>
+          <t>LinkedIn / Public</t>
         </is>
       </c>
       <c r="E25" s="16" t="inlineStr">
         <is>
-          <t>Auth. ₹30 Cr; paid-up ₹26.5 Cr; no external equity funding rounds identified</t>
+          <t>662 employees primarily engineering/manufacturing; limited visible software or data role hiring</t>
         </is>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>FIN06</t>
+          <t>SC02</t>
         </is>
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>Employee Productivity</t>
+          <t>Technical Workforce Depth</t>
         </is>
       </c>
       <c r="D26" s="16" t="inlineStr">
         <is>
-          <t>Tracxn</t>
+          <t>Tracxn / ICRA</t>
         </is>
       </c>
       <c r="E26" s="16" t="inlineStr">
         <is>
-          <t>662 employees; ₹531 Cr revenue = ~₹80 lakh revenue per employee</t>
+          <t>Strong mechanical and manufacturing engineering base; DSIR R&amp;D team; CNC and automation specialists</t>
         </is>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="B27" s="15" t="inlineStr">
         <is>
-          <t>IC01</t>
+          <t>SC03</t>
         </is>
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>Market Size</t>
+          <t>Digital Training Programs</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>IMARC Group 2024</t>
+          <t>Public records</t>
         </is>
       </c>
       <c r="E27" s="16" t="inlineStr">
         <is>
-          <t>India pneumatic equipment market $1.06B (2024) → $1.94B (2033)</t>
+          <t>No public L&amp;D investment, digital upskilling program, or online learning platform adoption disclosed</t>
         </is>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>IC02</t>
+          <t>SC04</t>
         </is>
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>Industry CAGR</t>
+          <t>Leadership Digital Literacy</t>
         </is>
       </c>
       <c r="D28" s="16" t="inlineStr">
         <is>
-          <t>IMARC Group</t>
+          <t>Janatics website / ICRA</t>
         </is>
       </c>
       <c r="E28" s="16" t="inlineStr">
         <is>
-          <t>India pneumatic equipment CAGR 6.9% (2025–2033)</t>
+          <t>Management I4.0 awareness demonstrated via product decisions; no digital leadership hire signals</t>
         </is>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1">
       <c r="B29" s="15" t="inlineStr">
         <is>
-          <t>IC03</t>
+          <t>SC05</t>
         </is>
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>Competitive Position</t>
+          <t>Innovation Culture Signals</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -3018,51 +2969,7 @@
       </c>
       <c r="E29" s="16" t="inlineStr">
         <is>
-          <t>Competes with SMC, Festo, Parker Hannifin; dominant domestic brand in mid-market</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="28" customHeight="1">
-      <c r="B30" s="15" t="inlineStr">
-        <is>
-          <t>IC04</t>
-        </is>
-      </c>
-      <c r="C30" s="16" t="inlineStr">
-        <is>
-          <t>Macro Tailwinds</t>
-        </is>
-      </c>
-      <c r="D30" s="16" t="inlineStr">
-        <is>
-          <t>Industry reports</t>
-        </is>
-      </c>
-      <c r="E30" s="16" t="inlineStr">
-        <is>
-          <t>Make in India, PLI for manufacturing, China+1 sourcing shifts — all favourable</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="B31" s="15" t="inlineStr">
-        <is>
-          <t>IC05</t>
-        </is>
-      </c>
-      <c r="C31" s="16" t="inlineStr">
-        <is>
-          <t>End-Market Mix</t>
-        </is>
-      </c>
-      <c r="D31" s="16" t="inlineStr">
-        <is>
-          <t>ICRA / Janatics</t>
-        </is>
-      </c>
-      <c r="E31" s="16" t="inlineStr">
-        <is>
-          <t>Pharma, auto, packaging, printing, food processing, medical equipment, textile — 7 sectors</t>
+          <t>DSIR R&amp;D present; no hackathon, innovation lab, startup engagement, or employee innovation program</t>
         </is>
       </c>
     </row>

</xml_diff>